<commit_message>
Add asset unit groups and courier login IDs
</commit_message>
<xml_diff>
--- a/public/templates/TEMPLATE_IMPORT_KENDARAAN_JNE.xlsx
+++ b/public/templates/TEMPLATE_IMPORT_KENDARAAN_JNE.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data" sheetId="1" r:id="R10f697144ad243b8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Petunjuk" sheetId="2" r:id="Raa08cdfc217a43d3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data" sheetId="1" r:id="R9851359515544acf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Petunjuk" sheetId="2" r:id="R9eecd03ab2c54ad5"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -241,15 +241,16 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="TemplateKendaraan" displayName="TemplateKendaraan" ref="A1:F3" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A1:F3"/>
-  <x:tableColumns count="6">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="TemplateKendaraan" displayName="TemplateKendaraan" ref="A1:G3" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A1:G3"/>
+  <x:tableColumns count="7">
     <x:tableColumn id="1" name="Kode Mobil"/>
     <x:tableColumn id="2" name="Plat Nomor"/>
     <x:tableColumn id="3" name="Jenis Kendaraan"/>
     <x:tableColumn id="4" name="KM Terakhir"/>
-    <x:tableColumn id="5" name="Status"/>
-    <x:tableColumn id="6" name="Keterangan"/>
+    <x:tableColumn id="5" name="Unit Aset"/>
+    <x:tableColumn id="6" name="Status"/>
+    <x:tableColumn id="7" name="Keterangan"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
@@ -454,8 +455,9 @@
     <x:col min="2" max="2" width="18" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="22" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="16" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="16" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="30" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="18" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="16" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="30" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="28" customHeight="1">
@@ -472,9 +474,12 @@
         <x:v>KM Terakhir</x:v>
       </x:c>
       <x:c r="E1" s="7" t="str">
+        <x:v>Unit Aset</x:v>
+      </x:c>
+      <x:c r="F1" s="7" t="str">
         <x:v>Status</x:v>
       </x:c>
-      <x:c r="F1" s="8" t="str">
+      <x:c r="G1" s="8" t="str">
         <x:v>Keterangan</x:v>
       </x:c>
     </x:row>
@@ -492,9 +497,12 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="E2" s="18" t="str">
+        <x:v>INBOUND</x:v>
+      </x:c>
+      <x:c r="F2" s="18" t="str">
         <x:v>AKTIF</x:v>
       </x:c>
-      <x:c r="F2" s="19" t="str">
+      <x:c r="G2" s="19" t="str">
         <x:v>Armada Tangerang</x:v>
       </x:c>
     </x:row>
@@ -512,9 +520,12 @@
         <x:v>12500</x:v>
       </x:c>
       <x:c r="E3" s="21" t="str">
+        <x:v>OUTBOUND</x:v>
+      </x:c>
+      <x:c r="F3" s="21" t="str">
         <x:v>AKTIF</x:v>
       </x:c>
-      <x:c r="F3" s="22" t="str">
+      <x:c r="G3" s="22" t="str">
         <x:v>Kendaraan sewa</x:v>
       </x:c>
     </x:row>
@@ -2010,14 +2021,17 @@
       <x:c r="D500" s="25"/>
     </x:row>
   </x:sheetData>
-  <x:dataValidations count="1">
+  <x:dataValidations count="2">
     <x:dataValidation type="list" sqref="E2:E500">
+      <x:formula1>"INBOUND,OUTBOUND"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="F2:F500">
       <x:formula1>"AKTIF,NONAKTIF"</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5913b2ee62a64b4f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R373f521b70d1498c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2056,22 +2070,22 @@
     </x:row>
     <x:row r="2" ht="26" customHeight="1">
       <x:c r="A2" s="30" t="str">
-        <x:v>JNE Mobile KM · Template Import Massal</x:v>
+        <x:v>Movetra · Template Import Massal</x:v>
       </x:c>
       <x:c r="B2" s="30" t="str">
-        <x:v>JNE Mobile KM · Template Import Massal</x:v>
+        <x:v>Movetra · Template Import Massal</x:v>
       </x:c>
       <x:c r="C2" s="30" t="str">
-        <x:v>JNE Mobile KM · Template Import Massal</x:v>
+        <x:v>Movetra · Template Import Massal</x:v>
       </x:c>
       <x:c r="D2" s="30" t="str">
-        <x:v>JNE Mobile KM · Template Import Massal</x:v>
+        <x:v>Movetra · Template Import Massal</x:v>
       </x:c>
       <x:c r="E2" s="30" t="str">
-        <x:v>JNE Mobile KM · Template Import Massal</x:v>
+        <x:v>Movetra · Template Import Massal</x:v>
       </x:c>
       <x:c r="F2" s="30" t="str">
-        <x:v>JNE Mobile KM · Template Import Massal</x:v>
+        <x:v>Movetra · Template Import Massal</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="30" customHeight="1">
@@ -2115,7 +2129,7 @@
         <x:v>4.</x:v>
       </x:c>
       <x:c r="B7" s="35" t="str">
-        <x:v>Status hanya boleh AKTIF atau NONAKTIF.</x:v>
+        <x:v>Unit Aset isi INBOUND atau OUTBOUND, atau nama unit lain yang sudah dibuat di Pengaturan Akun.</x:v>
       </x:c>
       <x:c r="C7" s="35"/>
       <x:c r="D7" s="35"/>
@@ -2127,12 +2141,24 @@
         <x:v>5.</x:v>
       </x:c>
       <x:c r="B8" s="35" t="str">
-        <x:v>Hapus baris contoh sebelum mengimpor data sebenarnya, lalu simpan sebagai XLSX atau CSV.</x:v>
+        <x:v>Status hanya boleh AKTIF atau NONAKTIF.</x:v>
       </x:c>
       <x:c r="C8" s="35"/>
       <x:c r="D8" s="35"/>
       <x:c r="E8" s="35"/>
       <x:c r="F8" s="35"/>
+    </x:row>
+    <x:row r="9" ht="30" customHeight="1">
+      <x:c r="A9" s="32" t="str">
+        <x:v>6.</x:v>
+      </x:c>
+      <x:c r="B9" s="35" t="str">
+        <x:v>Hapus baris contoh sebelum mengimpor data sebenarnya, lalu simpan sebagai XLSX atau CSV.</x:v>
+      </x:c>
+      <x:c r="C9" s="35"/>
+      <x:c r="D9" s="35"/>
+      <x:c r="E9" s="35"/>
+      <x:c r="F9" s="35"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -2143,6 +2169,7 @@
     <x:mergeCell ref="B6:F6"/>
     <x:mergeCell ref="B7:F7"/>
     <x:mergeCell ref="B8:F8"/>
+    <x:mergeCell ref="B9:F9"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>